<commit_message>
updated pizza bracekt with newest rating
</commit_message>
<xml_diff>
--- a/static/pizzaBracket/pizzaBracketRatings.xlsx
+++ b/static/pizzaBracket/pizzaBracketRatings.xlsx
@@ -1,21 +1,34 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29822"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29929"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/09258977402b9a53/Desktop/COOP/futureMath/personalWebsite/my-website/static/pizzaBracket/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="110" documentId="11_2BA3AA0112538A1F6E280854455DCE3A0743E58B" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{C7CE1EE5-1A9B-490A-8515-3F8860D6049A}"/>
+  <xr:revisionPtr revIDLastSave="169" documentId="11_2BA3AA0112538A1F6E280854455DCE3A0743E58B" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{A44B67AF-A268-4C29-8F35-DCA8054AB4D1}"/>
   <bookViews>
     <workbookView xWindow="-96" yWindow="-96" windowWidth="23232" windowHeight="12432" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Pizza Ratings" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="0"/>
+  <calcPr calcId="191029"/>
+  <extLst>
+    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
+      <xcalcf:calcFeatures>
+        <xcalcf:feature name="microsoft.com:RD"/>
+        <xcalcf:feature name="microsoft.com:Single"/>
+        <xcalcf:feature name="microsoft.com:FV"/>
+        <xcalcf:feature name="microsoft.com:CNMTM"/>
+        <xcalcf:feature name="microsoft.com:LET_WF"/>
+        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
+        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
+      </xcalcf:calcFeatures>
+    </ext>
+  </extLst>
 </workbook>
 </file>
 
@@ -91,21 +104,9 @@
     <t>(4) mama</t>
   </si>
   <si>
-    <t>(5) AK's</t>
-  </si>
-  <si>
     <t>(6) tremont house of pizza</t>
   </si>
   <si>
-    <t>Voter 12</t>
-  </si>
-  <si>
-    <t>Voter 13</t>
-  </si>
-  <si>
-    <t>Voter 14</t>
-  </si>
-  <si>
     <t>Voter 15</t>
   </si>
   <si>
@@ -140,6 +141,18 @@
   </si>
   <si>
     <t>Aidan</t>
+  </si>
+  <si>
+    <t>Alice</t>
+  </si>
+  <si>
+    <t>John</t>
+  </si>
+  <si>
+    <t>Ethan</t>
+  </si>
+  <si>
+    <t>(5) Crispy Dough</t>
   </si>
 </sst>
 </file>
@@ -280,6 +293,10 @@
     </ext>
   </extLst>
 </styleSheet>
+</file>
+
+<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
+<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -567,7 +584,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:U17"/>
+  <dimension ref="A1:U19"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.55000000000000004"/>
   <cols>
     <col min="1" max="1" width="12" customWidth="1"/>
@@ -696,21 +713,25 @@
         <v>22</v>
       </c>
       <c r="T2" s="9" t="s">
+        <v>39</v>
+      </c>
+      <c r="U2" s="9" t="s">
         <v>23</v>
-      </c>
-      <c r="U2" s="9" t="s">
-        <v>24</v>
       </c>
     </row>
     <row r="3" spans="1:21" x14ac:dyDescent="0.55000000000000004">
       <c r="A3" s="10" t="s">
-        <v>29</v>
+        <v>25</v>
       </c>
       <c r="B3" s="11"/>
       <c r="C3" s="11"/>
       <c r="D3" s="11"/>
-      <c r="E3" s="11"/>
-      <c r="F3" s="11"/>
+      <c r="E3" s="11">
+        <v>4</v>
+      </c>
+      <c r="F3" s="11">
+        <v>3</v>
+      </c>
       <c r="G3" s="11"/>
       <c r="H3" s="11"/>
       <c r="I3" s="11"/>
@@ -744,18 +765,26 @@
       <c r="S3" s="11">
         <v>4.8</v>
       </c>
-      <c r="T3" s="11"/>
-      <c r="U3" s="11"/>
+      <c r="T3" s="11">
+        <v>2</v>
+      </c>
+      <c r="U3" s="11">
+        <v>5</v>
+      </c>
     </row>
     <row r="4" spans="1:21" x14ac:dyDescent="0.55000000000000004">
       <c r="A4" s="10" t="s">
-        <v>30</v>
+        <v>26</v>
       </c>
       <c r="B4" s="11"/>
       <c r="C4" s="11"/>
       <c r="D4" s="11"/>
-      <c r="E4" s="11"/>
-      <c r="F4" s="11"/>
+      <c r="E4" s="11">
+        <v>4.5</v>
+      </c>
+      <c r="F4" s="11">
+        <v>3.5</v>
+      </c>
       <c r="G4" s="11"/>
       <c r="H4" s="11"/>
       <c r="I4" s="11"/>
@@ -789,18 +818,26 @@
       <c r="S4" s="11">
         <v>4</v>
       </c>
-      <c r="T4" s="11"/>
-      <c r="U4" s="11"/>
+      <c r="T4" s="11">
+        <v>5</v>
+      </c>
+      <c r="U4" s="11">
+        <v>3</v>
+      </c>
     </row>
     <row r="5" spans="1:21" x14ac:dyDescent="0.55000000000000004">
       <c r="A5" s="10" t="s">
-        <v>31</v>
+        <v>27</v>
       </c>
       <c r="B5" s="11"/>
       <c r="C5" s="11"/>
       <c r="D5" s="11"/>
-      <c r="E5" s="11"/>
-      <c r="F5" s="11"/>
+      <c r="E5" s="11">
+        <v>3</v>
+      </c>
+      <c r="F5" s="11">
+        <v>1.5</v>
+      </c>
       <c r="G5" s="11"/>
       <c r="H5" s="11"/>
       <c r="I5" s="11"/>
@@ -834,18 +871,26 @@
       <c r="S5" s="11">
         <v>4</v>
       </c>
-      <c r="T5" s="11"/>
-      <c r="U5" s="11"/>
+      <c r="T5" s="11">
+        <v>4.5</v>
+      </c>
+      <c r="U5" s="11">
+        <v>5</v>
+      </c>
     </row>
     <row r="6" spans="1:21" x14ac:dyDescent="0.55000000000000004">
       <c r="A6" s="10" t="s">
-        <v>32</v>
+        <v>28</v>
       </c>
       <c r="B6" s="11"/>
       <c r="C6" s="11"/>
       <c r="D6" s="11"/>
-      <c r="E6" s="11"/>
-      <c r="F6" s="11"/>
+      <c r="E6" s="11">
+        <v>4</v>
+      </c>
+      <c r="F6" s="11">
+        <v>4</v>
+      </c>
       <c r="G6" s="11"/>
       <c r="H6" s="11"/>
       <c r="I6" s="11"/>
@@ -879,18 +924,26 @@
       <c r="S6" s="11">
         <v>4</v>
       </c>
-      <c r="T6" s="11"/>
-      <c r="U6" s="11"/>
+      <c r="T6" s="11">
+        <v>5</v>
+      </c>
+      <c r="U6" s="11">
+        <v>2</v>
+      </c>
     </row>
     <row r="7" spans="1:21" x14ac:dyDescent="0.55000000000000004">
       <c r="A7" s="10" t="s">
-        <v>33</v>
+        <v>29</v>
       </c>
       <c r="B7" s="11"/>
       <c r="C7" s="11"/>
       <c r="D7" s="11"/>
-      <c r="E7" s="11"/>
-      <c r="F7" s="11"/>
+      <c r="E7" s="11">
+        <v>4</v>
+      </c>
+      <c r="F7" s="11">
+        <v>3.5</v>
+      </c>
       <c r="G7" s="11"/>
       <c r="H7" s="11"/>
       <c r="I7" s="11"/>
@@ -924,18 +977,26 @@
       <c r="S7" s="11">
         <v>3</v>
       </c>
-      <c r="T7" s="11"/>
-      <c r="U7" s="11"/>
+      <c r="T7" s="11">
+        <v>5</v>
+      </c>
+      <c r="U7" s="11">
+        <v>2</v>
+      </c>
     </row>
     <row r="8" spans="1:21" x14ac:dyDescent="0.55000000000000004">
       <c r="A8" s="10" t="s">
-        <v>34</v>
+        <v>30</v>
       </c>
       <c r="B8" s="11"/>
       <c r="C8" s="11"/>
       <c r="D8" s="11"/>
-      <c r="E8" s="11"/>
-      <c r="F8" s="11"/>
+      <c r="E8" s="11">
+        <v>1.5</v>
+      </c>
+      <c r="F8" s="11">
+        <v>1</v>
+      </c>
       <c r="G8" s="11"/>
       <c r="H8" s="11"/>
       <c r="I8" s="11"/>
@@ -955,18 +1016,26 @@
       <c r="Q8" s="11"/>
       <c r="R8" s="11"/>
       <c r="S8" s="11"/>
-      <c r="T8" s="11"/>
-      <c r="U8" s="11"/>
+      <c r="T8" s="11">
+        <v>5</v>
+      </c>
+      <c r="U8" s="11">
+        <v>2</v>
+      </c>
     </row>
     <row r="9" spans="1:21" x14ac:dyDescent="0.55000000000000004">
       <c r="A9" s="10" t="s">
-        <v>35</v>
+        <v>31</v>
       </c>
       <c r="B9" s="11"/>
       <c r="C9" s="11"/>
       <c r="D9" s="11"/>
-      <c r="E9" s="11"/>
-      <c r="F9" s="11"/>
+      <c r="E9" s="11">
+        <v>2.1</v>
+      </c>
+      <c r="F9" s="11">
+        <v>2</v>
+      </c>
       <c r="G9" s="11"/>
       <c r="H9" s="11"/>
       <c r="I9" s="11"/>
@@ -992,18 +1061,26 @@
       <c r="S9" s="11">
         <v>4</v>
       </c>
-      <c r="T9" s="11"/>
-      <c r="U9" s="11"/>
+      <c r="T9" s="11">
+        <v>5</v>
+      </c>
+      <c r="U9" s="11">
+        <v>4</v>
+      </c>
     </row>
     <row r="10" spans="1:21" x14ac:dyDescent="0.55000000000000004">
       <c r="A10" s="10" t="s">
-        <v>37</v>
+        <v>33</v>
       </c>
       <c r="B10" s="11"/>
       <c r="C10" s="11"/>
       <c r="D10" s="11"/>
-      <c r="E10" s="11"/>
-      <c r="F10" s="11"/>
+      <c r="E10" s="11">
+        <v>4</v>
+      </c>
+      <c r="F10" s="11">
+        <v>3.8</v>
+      </c>
       <c r="G10" s="11"/>
       <c r="H10" s="11"/>
       <c r="I10" s="11"/>
@@ -1037,12 +1114,16 @@
       <c r="S10" s="11">
         <v>3</v>
       </c>
-      <c r="T10" s="11"/>
-      <c r="U10" s="11"/>
+      <c r="T10" s="11">
+        <v>5</v>
+      </c>
+      <c r="U10" s="11">
+        <v>2</v>
+      </c>
     </row>
     <row r="11" spans="1:21" x14ac:dyDescent="0.55000000000000004">
       <c r="A11" s="10" t="s">
-        <v>38</v>
+        <v>34</v>
       </c>
       <c r="B11" s="11"/>
       <c r="C11" s="11"/>
@@ -1087,13 +1168,17 @@
     </row>
     <row r="12" spans="1:21" x14ac:dyDescent="0.55000000000000004">
       <c r="A12" s="10" t="s">
-        <v>39</v>
+        <v>35</v>
       </c>
       <c r="B12" s="11"/>
       <c r="C12" s="11"/>
       <c r="D12" s="11"/>
-      <c r="E12" s="11"/>
-      <c r="F12" s="11"/>
+      <c r="E12" s="11">
+        <v>3</v>
+      </c>
+      <c r="F12" s="11">
+        <v>5</v>
+      </c>
       <c r="G12" s="11"/>
       <c r="H12" s="11"/>
       <c r="I12" s="11"/>
@@ -1115,12 +1200,16 @@
       <c r="Q12" s="11"/>
       <c r="R12" s="11"/>
       <c r="S12" s="11"/>
-      <c r="T12" s="11"/>
-      <c r="U12" s="11"/>
+      <c r="T12" s="11">
+        <v>4</v>
+      </c>
+      <c r="U12" s="11">
+        <v>1</v>
+      </c>
     </row>
     <row r="13" spans="1:21" x14ac:dyDescent="0.55000000000000004">
       <c r="A13" s="10" t="s">
-        <v>36</v>
+        <v>32</v>
       </c>
       <c r="B13" s="11"/>
       <c r="C13" s="11"/>
@@ -1151,13 +1240,17 @@
     </row>
     <row r="14" spans="1:21" x14ac:dyDescent="0.55000000000000004">
       <c r="A14" s="10" t="s">
-        <v>25</v>
+        <v>36</v>
       </c>
       <c r="B14" s="11"/>
       <c r="C14" s="11"/>
       <c r="D14" s="11"/>
-      <c r="E14" s="11"/>
-      <c r="F14" s="11"/>
+      <c r="E14" s="11">
+        <v>3</v>
+      </c>
+      <c r="F14" s="11">
+        <v>1</v>
+      </c>
       <c r="G14" s="11"/>
       <c r="H14" s="11"/>
       <c r="I14" s="11"/>
@@ -1171,18 +1264,26 @@
       <c r="Q14" s="11"/>
       <c r="R14" s="11"/>
       <c r="S14" s="11"/>
-      <c r="T14" s="11"/>
-      <c r="U14" s="11"/>
+      <c r="T14" s="11">
+        <v>5</v>
+      </c>
+      <c r="U14" s="11">
+        <v>4</v>
+      </c>
     </row>
     <row r="15" spans="1:21" x14ac:dyDescent="0.55000000000000004">
       <c r="A15" s="10" t="s">
-        <v>26</v>
+        <v>37</v>
       </c>
       <c r="B15" s="11"/>
       <c r="C15" s="11"/>
       <c r="D15" s="11"/>
-      <c r="E15" s="11"/>
-      <c r="F15" s="11"/>
+      <c r="E15" s="11">
+        <v>1</v>
+      </c>
+      <c r="F15" s="11">
+        <v>3</v>
+      </c>
       <c r="G15" s="11"/>
       <c r="H15" s="11"/>
       <c r="I15" s="11"/>
@@ -1196,18 +1297,26 @@
       <c r="Q15" s="11"/>
       <c r="R15" s="11"/>
       <c r="S15" s="11"/>
-      <c r="T15" s="11"/>
-      <c r="U15" s="11"/>
+      <c r="T15" s="11">
+        <v>5</v>
+      </c>
+      <c r="U15" s="11">
+        <v>2</v>
+      </c>
     </row>
     <row r="16" spans="1:21" x14ac:dyDescent="0.55000000000000004">
       <c r="A16" s="10" t="s">
-        <v>27</v>
+        <v>38</v>
       </c>
       <c r="B16" s="11"/>
       <c r="C16" s="11"/>
       <c r="D16" s="11"/>
-      <c r="E16" s="11"/>
-      <c r="F16" s="11"/>
+      <c r="E16" s="11">
+        <v>3</v>
+      </c>
+      <c r="F16" s="11">
+        <v>4</v>
+      </c>
       <c r="G16" s="11"/>
       <c r="H16" s="11"/>
       <c r="I16" s="11"/>
@@ -1221,12 +1330,16 @@
       <c r="Q16" s="11"/>
       <c r="R16" s="11"/>
       <c r="S16" s="11"/>
-      <c r="T16" s="11"/>
-      <c r="U16" s="11"/>
+      <c r="T16" s="11">
+        <v>5</v>
+      </c>
+      <c r="U16" s="11">
+        <v>3.5</v>
+      </c>
     </row>
     <row r="17" spans="1:21" x14ac:dyDescent="0.55000000000000004">
       <c r="A17" s="10" t="s">
-        <v>28</v>
+        <v>24</v>
       </c>
       <c r="B17" s="11"/>
       <c r="C17" s="11"/>
@@ -1249,6 +1362,16 @@
       <c r="T17" s="11"/>
       <c r="U17" s="11"/>
     </row>
+    <row r="19" spans="1:21" x14ac:dyDescent="0.55000000000000004">
+      <c r="T19">
+        <f>AVERAGE(T3:T17)</f>
+        <v>4.625</v>
+      </c>
+      <c r="U19">
+        <f>AVERAGE(U3:U17)</f>
+        <v>2.9583333333333335</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
updated pizza bracket and created temp advising and research pages
</commit_message>
<xml_diff>
--- a/static/pizzaBracket/pizzaBracketRatings.xlsx
+++ b/static/pizzaBracket/pizzaBracketRatings.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/09258977402b9a53/Desktop/COOP/futureMath/personalWebsite/my-website/static/pizzaBracket/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="169" documentId="11_2BA3AA0112538A1F6E280854455DCE3A0743E58B" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{A44B67AF-A268-4C29-8F35-DCA8054AB4D1}"/>
+  <xr:revisionPtr revIDLastSave="171" documentId="11_2BA3AA0112538A1F6E280854455DCE3A0743E58B" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{A8385ED7-4E23-4781-832E-9F0111E78669}"/>
   <bookViews>
     <workbookView xWindow="-96" yWindow="-96" windowWidth="23232" windowHeight="12432" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -584,7 +584,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:U19"/>
+  <dimension ref="A1:U17"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.55000000000000004"/>
   <cols>
     <col min="1" max="1" width="12" customWidth="1"/>
@@ -1362,16 +1362,6 @@
       <c r="T17" s="11"/>
       <c r="U17" s="11"/>
     </row>
-    <row r="19" spans="1:21" x14ac:dyDescent="0.55000000000000004">
-      <c r="T19">
-        <f>AVERAGE(T3:T17)</f>
-        <v>4.625</v>
-      </c>
-      <c r="U19">
-        <f>AVERAGE(U3:U17)</f>
-        <v>2.9583333333333335</v>
-      </c>
-    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>